<commit_message>
The sample's code lists, each table's own (#248)
The arms in each table, SEX / AGEGR1 / RACE / ETHNIC in the demographics
tables (the CRF's values the data have none of print with 0), EOSSTT in
the disposition table; the variables sheet no longer says the order again.
T-14-1-1 and T-14-1-1S take 30 rows a page, to stay on one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/table_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/table_spec.xlsx
@@ -11,12 +11,13 @@
     <sheet name="variables" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="codelists" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="cells" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="layout" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="columns" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="style" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="cell_styles" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="col_header" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="about" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="digits" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="layout" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="columns" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="style" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="cell_styles" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="col_header" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="about" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -84,6 +85,159 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">The columns styled, | between them (.values = every value column); blank: every column.
+Example: Placebo | .values</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: TRUE styles the column header instead of the body; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">An R condition over the table's columns choosing the rows; blank: every row. Two rows with a where may not set the same look: join their conditions with |.
+Example: label == "Any TEAE"</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">left / center / right; blank: unchanged.
+Example: center</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Text colour, #RRGGBB; blank: unchanged.
+Example: #CC0000</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Cell shading, #RRGGBB; blank: unchanged.
+Example: #EEEEEE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Left indent of the cell text in twips (not on the header); blank: unchanged.
+Example: 200</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tflspec</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The report a row belongs to. Blank: a study-wide default; a row naming a report replaces the default row with the same key (ARD analyses: the report the analysis serves).
+Example: T-14-1-1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">The header row, a whole number (1 = the top).
 Example: 1</t>
         </r>
@@ -263,7 +417,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">With stats = rows: stat (the number) or stat_fmt (cards' formatted text) (plan_cells(value = )); blank: stat.
+          <t xml:space="preserve">Which of the ARD's values the table prints: stat (the number, rounded here: the digits sheet, a template's {x:.1f}) or stat_fmt (the ARD's own text, as it was formatted: no digits to set; a template still combines them, {mean} ({sd})); a row may say otherwise in its template ({mean:stat_fmt}, {mean:.1f}). With stats = rows: which goes in the cell (plan_cells(value = )). Blank: stat.
 Example: stat</t>
         </r>
       </text>
@@ -665,8 +819,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Rows a page (plan_paginate_rows(max_rows = )), a whole number; blank: as_rtftables()' default.
-Example: 26</t>
+          <t xml:space="preserve">Blank: every analysis variable (the rule); a variable: its exception.
+Example: WEIGHTBL</t>
         </r>
       </text>
     </comment>
@@ -678,8 +832,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">How a page break may cut: group_safe / group_force / rows / ... (plan_paginate_rows(split = )); blank: as_rtftables()' default.
-Example: group_force</t>
+          <t xml:space="preserve">The statistic, as the ARD names it (mean, sd, median, p ...).
+Example: mean</t>
         </r>
       </text>
     </comment>
@@ -691,332 +845,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Row positions to cut before, | between them, with pages_split = rows (plan_paginate_rows(break_before = )); blank: none.
-Example: 20 | 40</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Rows of a group kept together at the foot of a page, a whole number (plan_paginate_rows(min_group_rows = )); blank: the default.
-Example: 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Appended to a group label continued on the next page (plan_paginate_rows(cont_label = )); quote it to keep leading spaces; blank: none.
-Example: " (Cont.)"</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">BY pages: the column(s) whose value partitions the body first, each value a page, the row budget then applying within one (plan_paginate_rows(page_by = )); | between them; print it or hide it (columns$hide); blank: none.
-Example: APERIODC</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">With group_page = TRUE: the column whose values each start a page (plan_paginate_group(col = )); blank: the outermost row key.
-Example: PARAM</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">How groups print (plan_row_group(mode = )): value / indent / ...; blank: the default.
-Example: indent</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE, or the columns (names or positions, | between them) whose repeated values print once (plan_row_group(collapse = )); blank: none.
-Example: 1 | 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: one page per value of group_col (plan_paginate_group()); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: with group_page, FALSE leaves the group column unprinted (plan_paginate_group(keep = )); blank: TRUE.
-Example: FALSE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Where blank rows go: a named rule such as between_groups (plan_blanks(where = )); blank: none.
-Example: between_groups</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: a blank row before the first row (plan_blanks(first = )); blank: the default.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: a blank row after the last row (plan_blanks(last = )); blank: the default.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: blank rows count towards pages_max_rows (plan_blanks(counted = )); blank: the default.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The row-key columns folded into one stub column, | between them (plan_stub(vars = )); blank: the row keys.
-Example: group1 | label</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The stub column's name (plan_stub(name = )); blank: the default.
-Example: row_label</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Spaces a level is indented in the stub, a whole number (plan_stub(indent = )); blank: the default.
-Example: 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">How a group's summary row shows in the stub (plan_stub(group_summary = )); blank: the default.
-Example: header</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: fold the stub before cell styles and sorting see the rows (plan_stub(before = )); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Value columns a column page, a whole number (plan_paginate_cols(every = )); blank: no column pages.
-Example: 4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The columns to cut before (names or positions), | between them (plan_paginate_cols(at = )).
-Example: 16 | 29</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Columns printed on every column page (names or positions), | between them (plan_paginate_cols(keep = )); blank: the stub.
-Example: 1 | 2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The order the axes nest in, outermost first: group / rows / cols, or across / down (plan_paginate_cols(order = )); | between them; blank: the default.
-Example: across</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">A separator in the column names: one column page per key before it (plan_paginate_cols(cut_by = )).
-Example: ____</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: TRUE puts every column page on page 1's width scale, FALSE keeps each column's width (plan_paginate_cols(fit = )); blank: TRUE.
-Example: FALSE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: FALSE never cuts inside a spanning header cell (plan_paginate_cols(allow_span_break = )); blank: TRUE.
-Example: FALSE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">A column for people, on any sheet; never read. Any other column a sheet does not read is an error (a mistyped header).</t>
+          <t xml:space="preserve">Its decimals, a whole number (p, a percent: 1 prints 61.6).
+Example: 1</t>
         </r>
       </text>
     </comment>
@@ -1051,60 +881,358 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">A column name, or .values.
+          <t xml:space="preserve">Rows a page (plan_paginate_rows(max_rows = )), a whole number; blank: as_rtftables()' default.
+Example: 26</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">How a page break may cut: group_safe / group_force / rows / ... (plan_paginate_rows(split = )); blank: as_rtftables()' default.
+Example: group_force</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Row positions to cut before, | between them, with pages_split = rows (plan_paginate_rows(break_before = )); blank: none.
+Example: 20 | 40</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Rows of a group kept together at the foot of a page, a whole number (plan_paginate_rows(min_group_rows = )); blank: the default.
+Example: 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Appended to a group label continued on the next page (plan_paginate_rows(cont_label = )); quote it to keep leading spaces; blank: none.
+Example: " (Cont.)"</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">BY pages: the column(s) whose value partitions the body first, each value a page, the row budget then applying within one (plan_paginate_rows(page_by = )); | between them; print it or hide it (columns$hide); blank: none.
+Example: APERIODC</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">With group_page = TRUE: the column whose values each start a page (plan_paginate_group(col = )); blank: the outermost row key.
+Example: PARAM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">How groups print (plan_row_group(mode = )): value / indent / ...; blank: the default.
+Example: indent</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE, or the columns (names or positions, | between them) whose repeated values print once (plan_row_group(collapse = )); blank: none.
+Example: 1 | 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: one page per value of group_col (plan_paginate_group()); blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: with group_page, FALSE leaves the group column unprinted (plan_paginate_group(keep = )); blank: TRUE.
+Example: FALSE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Where blank rows go: a named rule such as between_groups (plan_blanks(where = )); blank: none.
+Example: between_groups</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: a blank row before the first row (plan_blanks(first = )); blank: the default.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: a blank row after the last row (plan_blanks(last = )); blank: the default.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: blank rows count towards pages_max_rows (plan_blanks(counted = )); blank: the default.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The row-key columns folded into one stub column, | between them (plan_stub(vars = )); blank: the row keys.
+Example: group1 | label</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The stub column's name (plan_stub(name = )); blank: the default.
 Example: row_label</t>
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Relative width (a number; plan_columns(widths = )). Give one to every printed column (.values covers the value columns); blank: rtfreporter's widths.
-Example: 5</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: a row-title column (plan_columns(row_title = )); blank: FALSE.
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Spaces a level is indented in the stub, a whole number (plan_stub(indent = )); blank: the default.
+Example: 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">How a group's summary row shows in the stub (plan_stub(group_summary = )); blank: the default.
+Example: header</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: fold the stub before cell styles and sorting see the rows (plan_stub(before = )); blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: align the decimal points (plan_columns(decimal = )); blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: used, not printed (plan_hide()); blank: FALSE.
-Example: TRUE</t>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Value columns a column page, a whole number (plan_paginate_cols(every = )); blank: no column pages.
+Example: 4</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The columns to cut before (names or positions), | between them (plan_paginate_cols(at = )).
+Example: 16 | 29</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Columns printed on every column page (names or positions), | between them (plan_paginate_cols(keep = )); blank: the stub.
+Example: 1 | 2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The order the axes nest in, outermost first: group / rows / cols, or across / down (plan_paginate_cols(order = )); | between them; blank: the default.
+Example: across</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">A separator in the column names: one column page per key before it (plan_paginate_cols(cut_by = )).
+Example: ____</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: TRUE puts every column page on page 1's width scale, FALSE keeps each column's width (plan_paginate_cols(fit = )); blank: TRUE.
+Example: FALSE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: FALSE never cuts inside a spanning header cell (plan_paginate_cols(allow_span_break = )); blank: TRUE.
+Example: FALSE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">A column for people, on any sheet; never read. Any other column a sheet does not read is an error (a mistyped header).</t>
         </r>
       </text>
     </comment>
@@ -1139,8 +1267,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The table's rules: tfl (header top and bottom, a bottom rule on the last row) or none; blank: tfl.
-Example: tfl</t>
+          <t xml:space="preserve">A column name, or .values.
+Example: row_label</t>
         </r>
       </text>
     </comment>
@@ -1152,37 +1280,37 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE: realign n (xx.x) count / percent cells to one width; blank: FALSE.
+          <t xml:space="preserve">Relative width (a number; plan_columns(widths = )). Give one to every printed column (.values covers the value columns); blank: rtfreporter's widths.
+Example: 5</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: a row-title column (plan_columns(row_title = )); blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: size each column to its widest content (plan_columns(auto_width = )); an explicit rel_width wins; blank: FALSE.
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: align the decimal points (plan_columns(decimal = )); blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Data row height in twips (1/1440 inch); blank: from the font size.
-Example: 240</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <r>
@@ -1191,346 +1319,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE: TRUE exact (clipped), FALSE at least; blank: FALSE.
+          <t xml:space="preserve">TRUE / FALSE: used, not printed (plan_hide()); blank: FALSE.
 Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Column-header row height in twips; blank: row_height_twips.
-Example: 300</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Blank separator row height in twips; blank: row_height_twips.
-Example: 120</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Left cell padding in twips; blank: 0.
-Example: 60</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Right cell padding in twips; blank: 0.
-Example: 60</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Font family of the table; blank: the document's (Courier).
-Example: Arial</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Font size in half-points (18 = 9 pt); blank: the document's.
-Example: 16</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Placement of the table: left / center / right; blank: left.
-Example: center</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Vertical alignment in a cell: bottom / top / center; blank: bottom.
-Example: top</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Cell-text markup, one of script (^{} _{} as super / subscript), relational (&gt;= &lt;= as symbols), all, none; blank: the document's (script).
-Example: all</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">One of detect (an all-empty data row prints as one blank row), collapse (a run of blank rows prints as one), none; blank: both detect and collapse.
-Example: none</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The column header's rules: sides from top | bottom | left | right, or none; blank: border's.
-Example: top | bottom</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The spanning header cells' rules: sides, or none; blank: border's.
-Example: bottom</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The body rows' rules: sides, or none; blank: border's.
-Example: none</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The first body row's rules: sides, or none; blank: border's.
-Example: top</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The last body row's rules: sides, or none; blank: border's.
-Example: bottom</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The whole column header's alignment: left / center / right (rtf_table_style()); blank: each column's.
-Example: center</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: the whole column header bold; blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: the whole column header italic; blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The body's default alignment: left / center / right (rtf_table_style()); blank: row-title columns left, the others center.
-Example: left</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: the body bold by default; blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: the body italic by default; blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE: the body underlined by default; blank: FALSE.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The table's width in twips (1/1440 inch); blank: the page's writable width.
-Example: 12960</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The table's width as a percentage of the page width; blank: the page's writable width.
-Example: 80</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The table's width as a percentage of the writable width (inside the margins); blank: 100.
-Example: 90</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">The column header text's alignment, every header row: left / center / right (plan_col_header(col_header_align = )); blank: each column's data alignment.
-Example: center</t>
         </r>
       </text>
     </comment>
@@ -1565,8 +1355,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The columns styled, | between them (.values = every value column); blank: every column.
-Example: Placebo | .values</t>
+          <t xml:space="preserve">The table's rules: tfl (header top and bottom, a bottom rule on the last row) or none; blank: tfl.
+Example: tfl</t>
         </r>
       </text>
     </comment>
@@ -1578,7 +1368,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE: TRUE styles the column header instead of the body; blank: FALSE.
+          <t xml:space="preserve">TRUE / FALSE: realign n (xx.x) count / percent cells to one width; blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
@@ -1591,8 +1381,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">An R condition over the table's columns choosing the rows; blank: every row. Two rows with a where may not set the same look: join their conditions with |.
-Example: label == "Any TEAE"</t>
+          <t xml:space="preserve">TRUE / FALSE: size each column to its widest content (plan_columns(auto_width = )); an explicit rel_width wins; blank: FALSE.
+Example: TRUE</t>
         </r>
       </text>
     </comment>
@@ -1604,86 +1394,359 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+          <t xml:space="preserve">Data row height in twips (1/1440 inch); blank: from the font size.
+Example: 240</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: TRUE exact (clipped), FALSE at least; blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Column-header row height in twips; blank: row_height_twips.
+Example: 300</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Blank separator row height in twips; blank: row_height_twips.
+Example: 120</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Left cell padding in twips; blank: 0.
+Example: 60</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Right cell padding in twips; blank: 0.
+Example: 60</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Font family of the table; blank: the document's (Courier).
+Example: Arial</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Font size in half-points (18 = 9 pt); blank: the document's.
+Example: 16</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Placement of the table: left / center / right; blank: left.
+Example: center</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Vertical alignment in a cell: bottom / top / center; blank: bottom.
+Example: top</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Cell-text markup, one of script (^{} _{} as super / subscript), relational (&gt;= &lt;= as symbols), all, none; blank: the document's (script).
+Example: all</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">One of detect (an all-empty data row prints as one blank row), collapse (a run of blank rows prints as one), none; blank: both detect and collapse.
+Example: none</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The column header's rules: sides from top | bottom | left | right, or none; blank: border's.
+Example: top | bottom</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The spanning header cells' rules: sides, or none; blank: border's.
+Example: bottom</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The body rows' rules: sides, or none; blank: border's.
+Example: none</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The first body row's rules: sides, or none; blank: border's.
+Example: top</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The last body row's rules: sides, or none; blank: border's.
+Example: bottom</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The whole column header's alignment: left / center / right (rtf_table_style()); blank: each column's.
+Example: center</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the whole column header bold; blank: FALSE.
 Example: TRUE</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">left / center / right; blank: unchanged.
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the whole column header italic; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The body's default alignment: left / center / right (rtf_table_style()); blank: row-title columns left, the others center.
+Example: left</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the body bold by default; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the body italic by default; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">TRUE / FALSE: the body underlined by default; blank: FALSE.
+Example: TRUE</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The table's width in twips (1/1440 inch); blank: the page's writable width.
+Example: 12960</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The table's width as a percentage of the page width; blank: the page's writable width.
+Example: 80</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The table's width as a percentage of the writable width (inside the margins); blank: 100.
+Example: 90</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The column header text's alignment, every header row: left / center / right (plan_col_header(col_header_align = )); blank: each column's data alignment.
 Example: center</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Text colour, #RRGGBB; blank: unchanged.
-Example: #CC0000</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Cell shading, #RRGGBB; blank: unchanged.
-Example: #EEEEEE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">TRUE / FALSE; blank: unchanged.
-Example: TRUE</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Left indent of the cell text in twips (not on the header); blank: unchanged.
-Example: 200</t>
         </r>
       </text>
     </comment>
@@ -1692,7 +1755,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="214">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1802,9 +1865,6 @@
     <t xml:space="preserve">empty_levels</t>
   </si>
   <si>
-    <t xml:space="preserve">Placebo | Xanomeline Low Dose | Xanomeline High Dose</t>
-  </si>
-  <si>
     <t xml:space="preserve">AGE</t>
   </si>
   <si>
@@ -1817,18 +1877,12 @@
     <t xml:space="preserve">Age group, n (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">18-64 | &gt;64</t>
-  </si>
-  <si>
     <t xml:space="preserve">SEX</t>
   </si>
   <si>
     <t xml:space="preserve">Sex, n (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">F | M</t>
-  </si>
-  <si>
     <t xml:space="preserve">RACE</t>
   </si>
   <si>
@@ -1847,9 +1901,6 @@
     <t xml:space="preserve">Status at end of study, n (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">COMPLETED | DISCONTINUED</t>
-  </si>
-  <si>
     <t xml:space="preserve">BASE</t>
   </si>
   <si>
@@ -1880,6 +1931,105 @@
     <t xml:space="preserve">Event-free probability (95% CI)</t>
   </si>
   <si>
+    <t xml:space="preserve">Placebo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xanomeline Low Dose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xanomeline High Dose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-64 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;64 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WHITE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLACK OR AFRICAN AMERICAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black or African American</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASIAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMERICAN INDIAN OR ALASKA NATIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">American Indian or Alaska Native</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NATIVE HAWAIIAN OR OTHER PACIFIC ISLANDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Native Hawaiian or Other Pacific Islander</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HISPANIC OR LATINO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hispanic or Latino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT HISPANIC OR LATINO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not Hispanic or Latino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT REPORTED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not reported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNKNOWN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPLETED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISCONTINUED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discontinued</t>
+  </si>
+  <si>
     <t xml:space="preserve">context</t>
   </si>
   <si>
@@ -1970,6 +2120,9 @@
     <t xml:space="preserve">1,1</t>
   </si>
   <si>
+    <t xml:space="preserve">statistic</t>
+  </si>
+  <si>
     <t xml:space="preserve">pages_max_rows</t>
   </si>
   <si>
@@ -2063,13 +2216,13 @@
     <t xml:space="preserve">study default</t>
   </si>
   <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">group_safe</t>
+  </si>
+  <si>
     <t xml:space="preserve">24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">group_safe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30</t>
   </si>
   <si>
     <t xml:space="preserve">22</t>
@@ -2608,249 +2761,35 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>172</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>197</v>
       </c>
       <c r="D1" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="E1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="F1" t="s">
-        <v>159</v>
+        <v>191</v>
       </c>
       <c r="G1" t="s">
-        <v>160</v>
+        <v>189</v>
       </c>
       <c r="H1" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="I1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2"/>
-      <c r="B2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-    </row>
-    <row r="3">
-      <c r="A3"/>
-      <c r="B3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E3" t="s">
-        <v>178</v>
-      </c>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
-    </row>
-    <row r="4">
-      <c r="A4"/>
-      <c r="B4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" t="s">
-        <v>121</v>
-      </c>
-      <c r="D4"/>
-      <c r="E4" t="s">
-        <v>179</v>
-      </c>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-    </row>
-    <row r="5">
-      <c r="A5"/>
-      <c r="B5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D5" t="s">
-        <v>177</v>
-      </c>
-      <c r="E5" t="s">
-        <v>180</v>
-      </c>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
-      <c r="I5"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6"/>
-      <c r="H6"/>
-      <c r="I6"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" t="s">
-        <v>134</v>
-      </c>
-      <c r="D7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E7" t="s">
-        <v>181</v>
-      </c>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C8" t="s">
-        <v>121</v>
-      </c>
-      <c r="D8"/>
-      <c r="E8" t="s">
-        <v>182</v>
-      </c>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" t="s">
-        <v>134</v>
-      </c>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" t="s">
-        <v>121</v>
-      </c>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" t="s">
-        <v>134</v>
-      </c>
-      <c r="D11" t="s">
-        <v>177</v>
-      </c>
-      <c r="E11" t="s">
-        <v>178</v>
-      </c>
-      <c r="F11"/>
-      <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C12" t="s">
-        <v>121</v>
-      </c>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12"/>
-      <c r="H12"/>
-      <c r="I12"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" t="s">
-        <v>134</v>
-      </c>
-      <c r="D13" t="s">
-        <v>177</v>
-      </c>
-      <c r="E13" t="s">
-        <v>180</v>
-      </c>
-      <c r="F13"/>
-      <c r="G13"/>
-      <c r="H13"/>
-      <c r="I13"/>
+        <v>200</v>
+      </c>
+      <c r="J1" t="s">
+        <v>192</v>
+      </c>
+      <c r="K1" t="s">
+        <v>201</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2866,6 +2805,267 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F1" t="s">
+        <v>189</v>
+      </c>
+      <c r="G1" t="s">
+        <v>190</v>
+      </c>
+      <c r="H1" t="s">
+        <v>205</v>
+      </c>
+      <c r="I1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2"/>
+      <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+    </row>
+    <row r="4">
+      <c r="A4"/>
+      <c r="B4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4"/>
+      <c r="E4" t="s">
+        <v>209</v>
+      </c>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+    </row>
+    <row r="5">
+      <c r="A5"/>
+      <c r="B5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E5" t="s">
+        <v>210</v>
+      </c>
+      <c r="F5"/>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C8" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8"/>
+      <c r="E8" t="s">
+        <v>212</v>
+      </c>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" t="s">
+        <v>164</v>
+      </c>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
+      <c r="H10"/>
+      <c r="I10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D11" t="s">
+        <v>207</v>
+      </c>
+      <c r="E11" t="s">
+        <v>208</v>
+      </c>
+      <c r="F11"/>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+      <c r="H12"/>
+      <c r="I12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" t="s">
+        <v>164</v>
+      </c>
+      <c r="D13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E13" t="s">
+        <v>210</v>
+      </c>
+      <c r="F13"/>
+      <c r="G13"/>
+      <c r="H13"/>
+      <c r="I13"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -2874,10 +3074,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>183</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -3102,13 +3302,15 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2" t="s">
         <v>36</v>
       </c>
+      <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2"/>
       <c r="F2"/>
     </row>
     <row r="3">
@@ -3116,13 +3318,13 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3"/>
       <c r="F3"/>
@@ -3132,17 +3334,15 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="s">
-        <v>41</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="E4"/>
       <c r="F4"/>
     </row>
     <row r="5">
@@ -3156,11 +3356,9 @@
         <v>43</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="s">
-        <v>44</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E5"/>
       <c r="F5"/>
     </row>
     <row r="6">
@@ -3168,63 +3366,63 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
         <v>45</v>
       </c>
-      <c r="C6" t="s">
-        <v>46</v>
-      </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6"/>
       <c r="F6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
-        <v>48</v>
-      </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E7"/>
       <c r="F7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8" t="s">
-        <v>36</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8"/>
       <c r="F8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>51</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E9"/>
       <c r="F9"/>
     </row>
     <row r="10">
@@ -3232,24 +3430,26 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10"/>
-      <c r="D10"/>
-      <c r="E10" t="s">
-        <v>36</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10"/>
       <c r="F10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -3259,13 +3459,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
@@ -3275,177 +3475,83 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14"/>
-      <c r="D14"/>
-      <c r="E14" t="s">
-        <v>36</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14"/>
       <c r="F14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15"/>
-      <c r="D15"/>
-      <c r="E15" t="s">
-        <v>36</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15"/>
       <c r="F15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E16"/>
       <c r="F16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E17"/>
       <c r="F17"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18" t="s">
-        <v>36</v>
-      </c>
-      <c r="F18"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19"/>
-      <c r="F19"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="s">
-        <v>44</v>
-      </c>
-      <c r="F21"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" t="n">
-        <v>4</v>
-      </c>
-      <c r="E22"/>
-      <c r="F22"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" t="s">
-        <v>47</v>
-      </c>
-      <c r="C23" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" t="n">
-        <v>5</v>
-      </c>
-      <c r="E23"/>
-      <c r="F23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3476,6 +3582,752 @@
         <v>33</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4"/>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5"/>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6"/>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7"/>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8"/>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9"/>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10"/>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11"/>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12"/>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13"/>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14"/>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15"/>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16"/>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" t="s">
+        <v>76</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" t="s">
+        <v>81</v>
+      </c>
+      <c r="D27" t="s">
+        <v>82</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" t="s">
+        <v>86</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D32"/>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33"/>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34"/>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>31</v>
+      </c>
+      <c r="B36" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" t="s">
+        <v>66</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" t="s">
+        <v>67</v>
+      </c>
+      <c r="D38" t="s">
+        <v>68</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" t="s">
+        <v>69</v>
+      </c>
+      <c r="D39" t="s">
+        <v>70</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>31</v>
+      </c>
+      <c r="B40" t="s">
+        <v>42</v>
+      </c>
+      <c r="C40" t="s">
+        <v>71</v>
+      </c>
+      <c r="D40" t="s">
+        <v>72</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" t="s">
+        <v>74</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" t="s">
+        <v>42</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" t="s">
+        <v>76</v>
+      </c>
+      <c r="E42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" t="s">
+        <v>77</v>
+      </c>
+      <c r="D43" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" t="s">
+        <v>44</v>
+      </c>
+      <c r="C44" t="s">
+        <v>79</v>
+      </c>
+      <c r="D44" t="s">
+        <v>80</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>31</v>
+      </c>
+      <c r="B45" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" t="s">
+        <v>81</v>
+      </c>
+      <c r="D45" t="s">
+        <v>82</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C46" t="s">
+        <v>83</v>
+      </c>
+      <c r="D46" t="s">
+        <v>84</v>
+      </c>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>31</v>
+      </c>
+      <c r="B47" t="s">
+        <v>44</v>
+      </c>
+      <c r="C47" t="s">
+        <v>85</v>
+      </c>
+      <c r="D47" t="s">
+        <v>86</v>
+      </c>
+      <c r="E47" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -3496,22 +4348,22 @@
         <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="E1" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="F1" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="G1" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="H1" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="I1" t="s">
         <v>14</v>
@@ -3522,15 +4374,15 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="G2"/>
       <c r="H2"/>
@@ -3541,13 +4393,13 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="G3"/>
       <c r="H3"/>
@@ -3558,13 +4410,13 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -3577,12 +4429,12 @@
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6">
@@ -3590,18 +4442,18 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="G6" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -3611,18 +4463,18 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="G7" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="H7"/>
       <c r="I7"/>
@@ -3632,18 +4484,18 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="G8" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="H8"/>
       <c r="I8"/>
@@ -3653,18 +4505,18 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="G9" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
@@ -3674,18 +4526,18 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="G10" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H10"/>
       <c r="I10"/>
@@ -3695,18 +4547,18 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="G11" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="H11"/>
       <c r="I11"/>
@@ -3716,18 +4568,18 @@
         <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="G12" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
@@ -3737,18 +4589,18 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="E13"/>
       <c r="F13" t="s">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="G13" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="H13"/>
       <c r="I13"/>
@@ -3758,18 +4610,18 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="G14" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="H14"/>
       <c r="I14"/>
@@ -3779,18 +4631,18 @@
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="E15"/>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H15"/>
       <c r="I15"/>
@@ -3800,18 +4652,18 @@
         <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="G16" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H16"/>
       <c r="I16"/>
@@ -3821,18 +4673,18 @@
         <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="E17"/>
       <c r="F17" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="G17" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="H17"/>
       <c r="I17"/>
@@ -3842,18 +4694,18 @@
         <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="G18" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="H18"/>
       <c r="I18"/>
@@ -3863,18 +4715,18 @@
         <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="G19" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H19"/>
       <c r="I19"/>
@@ -3896,85 +4748,111 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" t="s">
+        <v>124</v>
       </c>
       <c r="E1" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="F1" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="G1" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="H1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="I1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="J1" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="K1" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="L1" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="M1" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="N1" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="O1" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="P1" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="Q1" t="s">
-        <v>107</v>
+        <v>137</v>
       </c>
       <c r="R1" t="s">
-        <v>108</v>
+        <v>138</v>
       </c>
       <c r="S1" t="s">
-        <v>109</v>
+        <v>139</v>
       </c>
       <c r="T1" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="U1" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="V1" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="W1" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="X1" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="Y1" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="Z1" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="AA1" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
       <c r="AB1" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="AC1" t="s">
         <v>14</v>
@@ -3994,25 +4872,25 @@
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="N2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="O2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="P2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="Q2"/>
       <c r="R2" t="s">
-        <v>121</v>
+        <v>151</v>
       </c>
       <c r="S2"/>
       <c r="T2"/>
       <c r="U2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="V2"/>
       <c r="W2"/>
@@ -4022,7 +4900,7 @@
       <c r="AA2"/>
       <c r="AB2"/>
       <c r="AC2" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
@@ -4030,10 +4908,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="C3" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -4067,7 +4945,7 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -4102,10 +4980,10 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="C5" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -4139,10 +5017,10 @@
         <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="C6" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -4176,10 +5054,10 @@
         <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="C7" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -4215,62 +5093,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E1" t="s">
-        <v>131</v>
-      </c>
-      <c r="F1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2"/>
-      <c r="B2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-    </row>
-    <row r="3">
-      <c r="A3"/>
-      <c r="B3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D3"/>
-      <c r="E3"/>
-      <c r="F3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-  <legacyDrawing r:id="rIdvml"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -4281,104 +5103,160 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="D1" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="E1" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="F1" t="s">
-        <v>140</v>
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2"/>
+      <c r="B2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" t="s">
+        <v>170</v>
       </c>
       <c r="G1" t="s">
-        <v>141</v>
+        <v>171</v>
       </c>
       <c r="H1" t="s">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="I1" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="J1" t="s">
-        <v>144</v>
+        <v>174</v>
       </c>
       <c r="K1" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="L1" t="s">
-        <v>146</v>
+        <v>176</v>
       </c>
       <c r="M1" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
       <c r="N1" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="O1" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="P1" t="s">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="Q1" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="R1" t="s">
-        <v>152</v>
+        <v>182</v>
       </c>
       <c r="S1" t="s">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="T1" t="s">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="U1" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="V1" t="s">
-        <v>156</v>
+        <v>186</v>
       </c>
       <c r="W1" t="s">
-        <v>157</v>
+        <v>187</v>
       </c>
       <c r="X1" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="Y1" t="s">
-        <v>159</v>
+        <v>189</v>
       </c>
       <c r="Z1" t="s">
-        <v>160</v>
+        <v>190</v>
       </c>
       <c r="AA1" t="s">
-        <v>161</v>
+        <v>191</v>
       </c>
       <c r="AB1" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="AC1" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="AD1" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="AE1" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="AF1" t="s">
-        <v>166</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -4415,51 +5293,4 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <legacyDrawing r:id="rIdvml"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>167</v>
-      </c>
-      <c r="D1" t="s">
-        <v>168</v>
-      </c>
-      <c r="E1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F1" t="s">
-        <v>161</v>
-      </c>
-      <c r="G1" t="s">
-        <v>159</v>
-      </c>
-      <c r="H1" t="s">
-        <v>169</v>
-      </c>
-      <c r="I1" t="s">
-        <v>170</v>
-      </c>
-      <c r="J1" t="s">
-        <v>162</v>
-      </c>
-      <c r="K1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-  <legacyDrawing r:id="rIdvml"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
The sample regenerated: T-14-1-5/6 with overall and tables$total, no stacked Total (28/28, every RTF byte-identical)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/table_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/table_spec.xlsx
@@ -495,6 +495,32 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">The heading of a Total column (plan_total()): the ARD's overall rows, its analyses run again without their by (analyses$overall), as one more column; its {n} is the study total. Blank: none.
+Example: Total</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Where the Total column goes among the column key's values: last or first; blank: last.
+Example: first</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">A column for people, on any sheet; never read. Any other column a sheet does not read is an error (a mistyped header).</t>
         </r>
       </text>
@@ -1768,7 +1794,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="253">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1812,6 +1838,12 @@
     <t xml:space="preserve">header_n</t>
   </si>
   <si>
+    <t xml:space="preserve">total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total_position</t>
+  </si>
+  <si>
     <t xml:space="preserve">note</t>
   </si>
   <si>
@@ -1875,6 +1907,9 @@
     <t xml:space="preserve">T-14-1-5</t>
   </si>
   <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
     <t xml:space="preserve">Race, its Asian sub-categories nested under Asian: one block</t>
   </si>
   <si>
@@ -2095,9 +2130,6 @@
   </si>
   <si>
     <t xml:space="preserve">Unknown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
   </si>
   <si>
     <t xml:space="preserve">CHINESE</t>
@@ -2888,31 +2920,31 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F1" t="s">
+        <v>228</v>
+      </c>
+      <c r="G1" t="s">
         <v>226</v>
       </c>
-      <c r="G1" t="s">
-        <v>224</v>
-      </c>
       <c r="H1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="I1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="J1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="K1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -2932,37 +2964,37 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="H1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="I1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2974,16 +3006,16 @@
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
@@ -2993,14 +3025,14 @@
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
@@ -3010,16 +3042,16 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F5"/>
       <c r="G5"/>
@@ -3028,13 +3060,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -3045,19 +3077,19 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D7" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E7" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F7"/>
       <c r="G7"/>
@@ -3066,17 +3098,17 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C8" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D8"/>
       <c r="E8" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F8"/>
       <c r="G8"/>
@@ -3085,13 +3117,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
@@ -3102,13 +3134,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C10" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -3119,13 +3151,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -3136,17 +3168,17 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C12" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D12"/>
       <c r="E12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F12"/>
       <c r="G12"/>
@@ -3155,17 +3187,17 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D13"/>
       <c r="E13" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F13"/>
       <c r="G13"/>
@@ -3174,13 +3206,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C14" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
@@ -3191,19 +3223,19 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C15" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D15" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E15" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F15"/>
       <c r="G15"/>
@@ -3212,13 +3244,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C16" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
@@ -3229,19 +3261,19 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C17" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D17" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E17" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F17"/>
       <c r="G17"/>
@@ -3270,10 +3302,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3324,16 +3356,22 @@
       <c r="L1" t="s">
         <v>14</v>
       </c>
+      <c r="M1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -3343,19 +3381,21 @@
       <c r="I2"/>
       <c r="J2"/>
       <c r="K2"/>
-      <c r="L2" t="s">
-        <v>18</v>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
         <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -3365,19 +3405,21 @@
       <c r="I3"/>
       <c r="J3"/>
       <c r="K3"/>
-      <c r="L3" t="s">
-        <v>20</v>
+      <c r="L3"/>
+      <c r="M3"/>
+      <c r="N3" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -3387,19 +3429,21 @@
       <c r="I4"/>
       <c r="J4"/>
       <c r="K4"/>
-      <c r="L4" t="s">
-        <v>22</v>
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -3409,19 +3453,21 @@
       <c r="I5"/>
       <c r="J5"/>
       <c r="K5"/>
-      <c r="L5" t="s">
-        <v>25</v>
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -3431,19 +3477,21 @@
       <c r="I6"/>
       <c r="J6"/>
       <c r="K6"/>
-      <c r="L6" t="s">
-        <v>28</v>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -3453,19 +3501,21 @@
       <c r="I7"/>
       <c r="J7"/>
       <c r="K7"/>
-      <c r="L7" t="s">
-        <v>31</v>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
@@ -3475,19 +3525,21 @@
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
-      <c r="L8" t="s">
-        <v>33</v>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
@@ -3498,18 +3550,22 @@
       <c r="J9"/>
       <c r="K9"/>
       <c r="L9" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="M9"/>
+      <c r="N9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -3522,16 +3578,20 @@
       <c r="L10" t="s">
         <v>37</v>
       </c>
+      <c r="M10"/>
+      <c r="N10" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -3541,45 +3601,49 @@
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
-      <c r="L11" t="s">
-        <v>39</v>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="N11" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
       <c r="H12" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
-      <c r="L12" t="s">
-        <v>44</v>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -3589,8 +3653,10 @@
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
-      <c r="L13" t="s">
-        <v>18</v>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -3610,33 +3676,33 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -3647,13 +3713,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -3664,13 +3730,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
@@ -3681,13 +3747,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -3698,13 +3764,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -3715,13 +3781,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -3732,13 +3798,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -3749,13 +3815,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -3766,13 +3832,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D10" t="n">
         <v>3</v>
@@ -3783,13 +3849,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -3800,13 +3866,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -3817,13 +3883,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D13" t="n">
         <v>2</v>
@@ -3834,13 +3900,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D14" t="n">
         <v>3</v>
@@ -3851,13 +3917,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
@@ -3868,13 +3934,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -3885,13 +3951,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
@@ -3902,13 +3968,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -3919,13 +3985,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -3936,13 +4002,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -3953,13 +4019,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D21" t="n">
         <v>1</v>
@@ -3970,10 +4036,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C22"/>
       <c r="D22" t="n">
@@ -3982,18 +4048,18 @@
       <c r="E22"/>
       <c r="F22"/>
       <c r="G22" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
@@ -4004,13 +4070,13 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D24" t="n">
         <v>2</v>
@@ -4021,13 +4087,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
@@ -4038,13 +4104,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -4055,13 +4121,13 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D27" t="n">
         <v>3</v>
@@ -4072,13 +4138,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B28" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D28" t="n">
         <v>4</v>
@@ -4089,13 +4155,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D29" t="n">
         <v>5</v>
@@ -4121,7 +4187,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -4130,18 +4196,18 @@
         <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="n">
@@ -4150,13 +4216,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="n">
@@ -4165,13 +4231,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="n">
@@ -4180,13 +4246,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D5"/>
       <c r="E5" t="n">
@@ -4195,13 +4261,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D6"/>
       <c r="E6" t="n">
@@ -4210,13 +4276,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D7"/>
       <c r="E7" t="n">
@@ -4225,13 +4291,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D8"/>
       <c r="E8" t="n">
@@ -4240,13 +4306,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D9"/>
       <c r="E9" t="n">
@@ -4255,13 +4321,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D10"/>
       <c r="E10" t="n">
@@ -4270,13 +4336,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D11"/>
       <c r="E11" t="n">
@@ -4285,13 +4351,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D12"/>
       <c r="E12" t="n">
@@ -4300,13 +4366,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D13"/>
       <c r="E13" t="n">
@@ -4315,13 +4381,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D14"/>
       <c r="E14" t="n">
@@ -4330,13 +4396,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D15"/>
       <c r="E15" t="n">
@@ -4345,13 +4411,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D16"/>
       <c r="E16" t="n">
@@ -4360,13 +4426,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D17"/>
       <c r="E17" t="n">
@@ -4375,13 +4441,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D18"/>
       <c r="E18" t="n">
@@ -4390,13 +4456,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D19"/>
       <c r="E19" t="n">
@@ -4405,13 +4471,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D20"/>
       <c r="E20" t="n">
@@ -4420,13 +4486,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D21"/>
       <c r="E21" t="n">
@@ -4435,13 +4501,13 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D22"/>
       <c r="E22" t="n">
@@ -4450,16 +4516,16 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4467,16 +4533,16 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D24" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4484,13 +4550,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="n">
@@ -4499,16 +4565,16 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
@@ -4516,16 +4582,16 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D27" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
@@ -4533,16 +4599,16 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
@@ -4550,16 +4616,16 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
@@ -4567,16 +4633,16 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
@@ -4584,16 +4650,16 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D31" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E31" t="n">
         <v>2</v>
@@ -4601,16 +4667,16 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C32" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E32" t="n">
         <v>3</v>
@@ -4618,16 +4684,16 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C33" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D33" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E33" t="n">
         <v>4</v>
@@ -4635,16 +4701,16 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D34" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E34" t="n">
         <v>5</v>
@@ -4652,16 +4718,16 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C35" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D35" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E35" t="n">
         <v>1</v>
@@ -4669,16 +4735,16 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C36" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D36" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -4686,16 +4752,16 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B37" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D37" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -4703,16 +4769,16 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B38" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C38" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>
@@ -4720,16 +4786,16 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B39" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C39" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D39" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -4737,16 +4803,16 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B40" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C40" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>
@@ -4754,16 +4820,16 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B41" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C41" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
@@ -4771,16 +4837,16 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B42" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C42" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E42" t="n">
         <v>2</v>
@@ -4788,16 +4854,16 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C43" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D43" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E43" t="n">
         <v>3</v>
@@ -4805,16 +4871,16 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C44" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D44" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E44" t="n">
         <v>4</v>
@@ -4822,16 +4888,16 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C45" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D45" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E45" t="n">
         <v>5</v>
@@ -4839,16 +4905,16 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D46" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E46" t="n">
         <v>1</v>
@@ -4856,16 +4922,16 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C47" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D47" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -4873,16 +4939,16 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B48" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C48" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D48" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E48" t="n">
         <v>3</v>
@@ -4890,16 +4956,16 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B49" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C49" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D49" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E49" t="n">
         <v>4</v>
@@ -4907,13 +4973,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B50" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C50" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D50"/>
       <c r="E50" t="n">
@@ -4922,13 +4988,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B51" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C51" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D51"/>
       <c r="E51" t="n">
@@ -4937,13 +5003,13 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B52" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C52" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D52"/>
       <c r="E52" t="n">
@@ -4952,13 +5018,13 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B53" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C53" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D53"/>
       <c r="E53" t="n">
@@ -4967,457 +5033,461 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B54" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C54" t="s">
-        <v>109</v>
-      </c>
-      <c r="D54"/>
+        <v>94</v>
+      </c>
+      <c r="D54" t="s">
+        <v>95</v>
+      </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B55" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C55" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D55" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B56" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C56" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D56" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B57" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C57" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D57" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B58" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C58" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D58" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B59" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="C59" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D59" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B60" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D60" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B61" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C61" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D61" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B62" t="s">
-        <v>76</v>
+        <v>32</v>
       </c>
       <c r="C62" t="s">
-        <v>114</v>
-      </c>
-      <c r="D62" t="s">
-        <v>115</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D62"/>
       <c r="E62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C63" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D63"/>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B64" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C64" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D64"/>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B65" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C65" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D65"/>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B66" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
-      </c>
-      <c r="D66"/>
+        <v>94</v>
+      </c>
+      <c r="D66" t="s">
+        <v>95</v>
+      </c>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B67" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C67" t="s">
-        <v>109</v>
-      </c>
-      <c r="D67"/>
+        <v>96</v>
+      </c>
+      <c r="D67" t="s">
+        <v>97</v>
+      </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B68" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C68" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D68" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B69" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C69" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="D69" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B70" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C70" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="D70" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B71" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="C71" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="D71" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="E71" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B72" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="C72" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="D72" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="E72" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B73" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C73" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D73" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B74" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="C74" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D74" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B75" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="C75" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D75" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="B76" t="s">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="C76" t="s">
-        <v>116</v>
-      </c>
-      <c r="D76" t="s">
-        <v>117</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D76"/>
       <c r="E76" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="B77" t="s">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="C77" t="s">
-        <v>118</v>
-      </c>
-      <c r="D77" t="s">
-        <v>119</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D77"/>
       <c r="E77" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B78" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C78" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D78"/>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B79" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="C79" t="s">
-        <v>80</v>
-      </c>
-      <c r="D79"/>
+        <v>85</v>
+      </c>
+      <c r="D79" t="s">
+        <v>86</v>
+      </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B80" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="C80" t="s">
-        <v>81</v>
-      </c>
-      <c r="D80"/>
+        <v>87</v>
+      </c>
+      <c r="D80" t="s">
+        <v>88</v>
+      </c>
       <c r="E80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B81" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C81" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E81" t="n">
         <v>1</v>
@@ -5425,16 +5495,16 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B82" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C82" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="D82" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E82" t="n">
         <v>2</v>
@@ -5442,16 +5512,16 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B83" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C83" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D83" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E83" t="n">
         <v>1</v>
@@ -5459,16 +5529,16 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B84" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C84" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D84" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="E84" t="n">
         <v>2</v>
@@ -5476,154 +5546,120 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B85" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C85" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D85" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B86" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C86" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="D86" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B87" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C87" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="D87" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B88" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C88" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D88" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B89" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C89" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D89" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B90" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C90" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="D90" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B91" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C91" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D91" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="s">
-        <v>45</v>
-      </c>
-      <c r="B92" t="s">
-        <v>59</v>
-      </c>
-      <c r="C92" t="s">
-        <v>105</v>
-      </c>
-      <c r="D92" t="s">
-        <v>106</v>
-      </c>
-      <c r="E92" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="s">
-        <v>45</v>
-      </c>
-      <c r="B93" t="s">
-        <v>59</v>
-      </c>
-      <c r="C93" t="s">
-        <v>107</v>
-      </c>
-      <c r="D93" t="s">
-        <v>108</v>
-      </c>
-      <c r="E93" t="n">
         <v>4</v>
       </c>
     </row>
@@ -5644,44 +5680,44 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G2"/>
       <c r="H2"/>
@@ -5689,16 +5725,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G3"/>
       <c r="H3"/>
@@ -5706,16 +5742,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -5728,234 +5764,234 @@
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H7"/>
       <c r="I7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H8"/>
       <c r="I8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H10"/>
       <c r="I10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H11"/>
       <c r="I11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E13"/>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H13"/>
       <c r="I13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H14"/>
       <c r="I14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E15"/>
       <c r="F15" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H15"/>
       <c r="I15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G16"/>
       <c r="H16"/>
@@ -5963,231 +5999,231 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E17"/>
       <c r="F17" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G17" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H17"/>
       <c r="I17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G18" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H18"/>
       <c r="I18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G19" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H19"/>
       <c r="I19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E20"/>
       <c r="F20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G20" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H20"/>
       <c r="I20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C21"/>
       <c r="D21" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E21"/>
       <c r="F21" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C22"/>
       <c r="D22" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E22"/>
       <c r="F22" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G22" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H22"/>
       <c r="I22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B23" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C23"/>
       <c r="D23" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E23"/>
       <c r="F23" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G23" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H23"/>
       <c r="I23"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C24"/>
       <c r="D24" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E24"/>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H24"/>
       <c r="I24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C25"/>
       <c r="D25" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E25"/>
       <c r="F25" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G25" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H25"/>
       <c r="I25"/>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C26"/>
       <c r="D26" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E26"/>
       <c r="F26" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G26" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H26"/>
       <c r="I26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B27" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C27"/>
       <c r="D27" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E27"/>
       <c r="F27" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H27"/>
       <c r="I27"/>
@@ -6209,13 +6245,13 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -6235,88 +6271,88 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="J1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="K1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="L1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="M1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="N1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="O1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="P1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="Q1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="R1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="S1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="T1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="V1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="W1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="X1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="Y1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Z1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AA1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="AB1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="AC1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
@@ -6333,25 +6369,25 @@
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="N2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="O2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="P2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="Q2"/>
       <c r="R2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="S2"/>
       <c r="T2"/>
       <c r="U2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="V2"/>
       <c r="W2"/>
@@ -6361,18 +6397,18 @@
       <c r="AA2"/>
       <c r="AB2"/>
       <c r="AC2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -6403,10 +6439,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -6438,13 +6474,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -6475,10 +6511,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -6510,13 +6546,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -6547,10 +6583,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -6582,10 +6618,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
@@ -6617,10 +6653,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
@@ -6652,10 +6688,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C11"/>
       <c r="D11"/>
@@ -6687,13 +6723,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C12" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
@@ -6724,13 +6760,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C13" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -6776,28 +6812,28 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -6806,10 +6842,10 @@
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -6832,104 +6868,104 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="K1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="L1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="M1" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="N1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="O1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="P1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="Q1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="R1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="S1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="T1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="U1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="V1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="W1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="X1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="Y1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="Z1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="AA1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="AB1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AC1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="AD1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="AE1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="AF1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>

</xml_diff>

<commit_message>
The generated programs, reviewed again (#347): report_id names the report, a study-folder check, a failed program's error kept, the sample's code lists and names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/table_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/table_spec.xlsx
@@ -1794,7 +1794,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -2051,6 +2051,9 @@
     <t xml:space="preserve">Xanomeline High Dose</t>
   </si>
   <si>
+    <t xml:space="preserve">F-14-2-4</t>
+  </si>
+  <si>
     <t xml:space="preserve">F</t>
   </si>
   <si>
@@ -2063,19 +2066,19 @@
     <t xml:space="preserve">Male</t>
   </si>
   <si>
+    <t xml:space="preserve">18-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-64 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;64 years</t>
+  </si>
+  <si>
     <t xml:space="preserve">Screen Failure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18-64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18-64 years</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;64 years</t>
   </si>
   <si>
     <t xml:space="preserve">WHITE</t>
@@ -2923,31 +2926,31 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F1" t="s">
+        <v>230</v>
+      </c>
+      <c r="G1" t="s">
         <v>228</v>
       </c>
-      <c r="F1" t="s">
-        <v>229</v>
-      </c>
-      <c r="G1" t="s">
-        <v>227</v>
-      </c>
       <c r="H1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -2967,37 +2970,37 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -3009,16 +3012,16 @@
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
@@ -3028,14 +3031,14 @@
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
@@ -3045,16 +3048,16 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F5"/>
       <c r="G5"/>
@@ -3066,10 +3069,10 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -3083,16 +3086,16 @@
         <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F7"/>
       <c r="G7"/>
@@ -3104,14 +3107,14 @@
         <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D8"/>
       <c r="E8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F8"/>
       <c r="G8"/>
@@ -3123,10 +3126,10 @@
         <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
@@ -3140,10 +3143,10 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -3157,10 +3160,10 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -3174,14 +3177,14 @@
         <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D12"/>
       <c r="E12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F12"/>
       <c r="G12"/>
@@ -3193,14 +3196,14 @@
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D13"/>
       <c r="E13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F13"/>
       <c r="G13"/>
@@ -3212,10 +3215,10 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
@@ -3229,16 +3232,16 @@
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F15"/>
       <c r="G15"/>
@@ -3250,10 +3253,10 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
@@ -3267,16 +3270,16 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D17" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F17"/>
       <c r="G17"/>
@@ -3305,10 +3308,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -4610,10 +4613,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C20" t="s">
         <v>82</v>
@@ -4625,10 +4628,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
         <v>83</v>
@@ -4640,10 +4643,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C22" t="s">
         <v>84</v>
@@ -4655,16 +4658,16 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="B23" t="s">
         <v>58</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -4672,16 +4675,16 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="B24" t="s">
         <v>58</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -4689,99 +4692,95 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
-      </c>
-      <c r="D25"/>
+        <v>90</v>
+      </c>
+      <c r="D25" t="s">
+        <v>91</v>
+      </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>85</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D26" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" t="s">
-        <v>88</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D27"/>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" t="s">
-        <v>91</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D28"/>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>92</v>
-      </c>
-      <c r="D29" t="s">
-        <v>93</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="D29"/>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="D30" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
@@ -4789,16 +4788,16 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="E31" t="n">
         <v>2</v>
@@ -4809,16 +4808,14 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C32" t="s">
-        <v>98</v>
-      </c>
-      <c r="D32" t="s">
-        <v>99</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D32"/>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -4826,16 +4823,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="D33" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -4843,21 +4840,21 @@
         <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="D34" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B35" t="s">
         <v>56</v>
@@ -4874,7 +4871,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B36" t="s">
         <v>56</v>
@@ -4891,16 +4888,16 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B37" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C37" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="D37" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -4908,16 +4905,16 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B38" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C38" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>
@@ -4925,87 +4922,87 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C39" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B40" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C40" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D40" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B41" t="s">
         <v>60</v>
       </c>
       <c r="C41" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="D41" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D42" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="B43" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C43" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D43" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -5013,16 +5010,16 @@
         <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C44" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="D44" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -5030,16 +5027,16 @@
         <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C45" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="D45" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -5047,13 +5044,13 @@
         <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C46" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D46" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="E46" t="n">
         <v>1</v>
@@ -5064,13 +5061,13 @@
         <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C47" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="D47" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -5081,16 +5078,16 @@
         <v>17</v>
       </c>
       <c r="B48" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C48" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="D48" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -5098,127 +5095,135 @@
         <v>17</v>
       </c>
       <c r="B49" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C49" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D49" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B50" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="C50" t="s">
-        <v>82</v>
-      </c>
-      <c r="D50"/>
+        <v>99</v>
+      </c>
+      <c r="D50" t="s">
+        <v>100</v>
+      </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B51" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="C51" t="s">
-        <v>83</v>
-      </c>
-      <c r="D51"/>
+        <v>101</v>
+      </c>
+      <c r="D51" t="s">
+        <v>102</v>
+      </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B52" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="C52" t="s">
-        <v>84</v>
-      </c>
-      <c r="D52"/>
+        <v>103</v>
+      </c>
+      <c r="D52" t="s">
+        <v>104</v>
+      </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B53" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="C53" t="s">
-        <v>89</v>
-      </c>
-      <c r="D53"/>
+        <v>105</v>
+      </c>
+      <c r="D53" t="s">
+        <v>106</v>
+      </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B54" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C54" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="D54" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B55" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C55" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="D55" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B56" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C56" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="D56" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57">
@@ -5226,16 +5231,14 @@
         <v>36</v>
       </c>
       <c r="B57" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>100</v>
-      </c>
-      <c r="D57" t="s">
-        <v>101</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D57"/>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -5243,16 +5246,14 @@
         <v>36</v>
       </c>
       <c r="B58" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C58" t="s">
-        <v>102</v>
-      </c>
-      <c r="D58" t="s">
-        <v>103</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D58"/>
       <c r="E58" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
@@ -5260,16 +5261,14 @@
         <v>36</v>
       </c>
       <c r="B59" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="C59" t="s">
-        <v>112</v>
-      </c>
-      <c r="D59" t="s">
-        <v>113</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="D59"/>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">
@@ -5277,16 +5276,14 @@
         <v>36</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="C60" t="s">
-        <v>114</v>
-      </c>
-      <c r="D60" t="s">
-        <v>115</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D60"/>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
@@ -5294,16 +5291,16 @@
         <v>36</v>
       </c>
       <c r="B61" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="C61" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="D61" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -5311,16 +5308,16 @@
         <v>36</v>
       </c>
       <c r="B62" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="D62" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -5328,16 +5325,16 @@
         <v>36</v>
       </c>
       <c r="B63" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C63" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D63" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
@@ -5345,16 +5342,16 @@
         <v>36</v>
       </c>
       <c r="B64" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C64" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D64" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -5362,16 +5359,16 @@
         <v>36</v>
       </c>
       <c r="B65" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C65" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D65" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
@@ -5379,13 +5376,13 @@
         <v>36</v>
       </c>
       <c r="B66" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="C66" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D66" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E66" t="n">
         <v>1</v>
@@ -5396,13 +5393,13 @@
         <v>36</v>
       </c>
       <c r="B67" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="C67" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="D67" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E67" t="n">
         <v>2</v>
@@ -5413,13 +5410,13 @@
         <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="C68" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="D68" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E68" t="n">
         <v>3</v>
@@ -5430,127 +5427,135 @@
         <v>36</v>
       </c>
       <c r="B69" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C69" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="D69" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="E69" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B70" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C70" t="s">
-        <v>82</v>
-      </c>
-      <c r="D70"/>
+        <v>88</v>
+      </c>
+      <c r="D70" t="s">
+        <v>89</v>
+      </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B71" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C71" t="s">
-        <v>83</v>
-      </c>
-      <c r="D71"/>
+        <v>90</v>
+      </c>
+      <c r="D71" t="s">
+        <v>91</v>
+      </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B72" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C72" t="s">
-        <v>84</v>
-      </c>
-      <c r="D72"/>
+        <v>92</v>
+      </c>
+      <c r="D72" t="s">
+        <v>93</v>
+      </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B73" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
-      </c>
-      <c r="D73"/>
+        <v>105</v>
+      </c>
+      <c r="D73" t="s">
+        <v>106</v>
+      </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B74" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C74" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="D74" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B75" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C75" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="D75" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B76" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C76" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="D76" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="E76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
@@ -5558,16 +5563,14 @@
         <v>39</v>
       </c>
       <c r="B77" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C77" t="s">
-        <v>100</v>
-      </c>
-      <c r="D77" t="s">
-        <v>101</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D77"/>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -5575,16 +5578,14 @@
         <v>39</v>
       </c>
       <c r="B78" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C78" t="s">
-        <v>102</v>
-      </c>
-      <c r="D78" t="s">
-        <v>103</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D78"/>
       <c r="E78" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
@@ -5592,16 +5593,14 @@
         <v>39</v>
       </c>
       <c r="B79" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="C79" t="s">
-        <v>112</v>
-      </c>
-      <c r="D79" t="s">
-        <v>113</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="D79"/>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
@@ -5609,16 +5608,14 @@
         <v>39</v>
       </c>
       <c r="B80" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="C80" t="s">
-        <v>114</v>
-      </c>
-      <c r="D80" t="s">
-        <v>115</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D80"/>
       <c r="E80" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
@@ -5626,16 +5623,16 @@
         <v>39</v>
       </c>
       <c r="B81" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="C81" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="D81" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="E81" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -5643,16 +5640,16 @@
         <v>39</v>
       </c>
       <c r="B82" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C82" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="D82" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
@@ -5660,16 +5657,16 @@
         <v>39</v>
       </c>
       <c r="B83" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C83" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D83" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84">
@@ -5677,16 +5674,16 @@
         <v>39</v>
       </c>
       <c r="B84" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C84" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D84" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
@@ -5694,16 +5691,16 @@
         <v>39</v>
       </c>
       <c r="B85" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C85" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D85" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="86">
@@ -5711,13 +5708,13 @@
         <v>39</v>
       </c>
       <c r="B86" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="C86" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D86" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E86" t="n">
         <v>1</v>
@@ -5728,13 +5725,13 @@
         <v>39</v>
       </c>
       <c r="B87" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="C87" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="D87" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E87" t="n">
         <v>2</v>
@@ -5745,13 +5742,13 @@
         <v>39</v>
       </c>
       <c r="B88" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="C88" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="D88" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E88" t="n">
         <v>3</v>
@@ -5762,143 +5759,149 @@
         <v>39</v>
       </c>
       <c r="B89" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C89" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="D89" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B90" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C90" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="D90" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B91" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C91" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="D91" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B92" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="C92" t="s">
-        <v>82</v>
-      </c>
-      <c r="D92"/>
+        <v>92</v>
+      </c>
+      <c r="D92" t="s">
+        <v>93</v>
+      </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B93" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="C93" t="s">
-        <v>83</v>
-      </c>
-      <c r="D93"/>
+        <v>105</v>
+      </c>
+      <c r="D93" t="s">
+        <v>106</v>
+      </c>
       <c r="E93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B94" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="C94" t="s">
-        <v>84</v>
-      </c>
-      <c r="D94"/>
+        <v>107</v>
+      </c>
+      <c r="D94" t="s">
+        <v>108</v>
+      </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B95" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C95" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="D95" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B96" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C96" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="D96" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="B97" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C97" t="s">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="D97" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="E97" t="n">
         <v>1</v>
@@ -5906,16 +5909,16 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="B98" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C98" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="D98" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="E98" t="n">
         <v>2</v>
@@ -5926,14 +5929,12 @@
         <v>48</v>
       </c>
       <c r="B99" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="C99" t="s">
-        <v>94</v>
-      </c>
-      <c r="D99" t="s">
-        <v>95</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D99"/>
       <c r="E99" t="n">
         <v>1</v>
       </c>
@@ -5943,14 +5944,12 @@
         <v>48</v>
       </c>
       <c r="B100" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="C100" t="s">
-        <v>96</v>
-      </c>
-      <c r="D100" t="s">
-        <v>97</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D100"/>
       <c r="E100" t="n">
         <v>2</v>
       </c>
@@ -5960,14 +5959,12 @@
         <v>48</v>
       </c>
       <c r="B101" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="C101" t="s">
-        <v>98</v>
-      </c>
-      <c r="D101" t="s">
-        <v>99</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="D101"/>
       <c r="E101" t="n">
         <v>3</v>
       </c>
@@ -5977,16 +5974,16 @@
         <v>48</v>
       </c>
       <c r="B102" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C102" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="D102" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="E102" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -5994,16 +5991,16 @@
         <v>48</v>
       </c>
       <c r="B103" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C103" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="D103" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="E103" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
@@ -6011,13 +6008,13 @@
         <v>48</v>
       </c>
       <c r="B104" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C104" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D104" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="E104" t="n">
         <v>1</v>
@@ -6028,13 +6025,13 @@
         <v>48</v>
       </c>
       <c r="B105" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C105" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="D105" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="E105" t="n">
         <v>2</v>
@@ -6045,16 +6042,16 @@
         <v>48</v>
       </c>
       <c r="B106" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C106" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="D106" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="E106" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -6062,15 +6059,134 @@
         <v>48</v>
       </c>
       <c r="B107" t="s">
+        <v>60</v>
+      </c>
+      <c r="C107" t="s">
+        <v>97</v>
+      </c>
+      <c r="D107" t="s">
+        <v>98</v>
+      </c>
+      <c r="E107" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>48</v>
+      </c>
+      <c r="B108" t="s">
+        <v>60</v>
+      </c>
+      <c r="C108" t="s">
+        <v>99</v>
+      </c>
+      <c r="D108" t="s">
+        <v>100</v>
+      </c>
+      <c r="E108" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>48</v>
+      </c>
+      <c r="B109" t="s">
+        <v>60</v>
+      </c>
+      <c r="C109" t="s">
+        <v>101</v>
+      </c>
+      <c r="D109" t="s">
+        <v>102</v>
+      </c>
+      <c r="E109" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>48</v>
+      </c>
+      <c r="B110" t="s">
+        <v>60</v>
+      </c>
+      <c r="C110" t="s">
+        <v>103</v>
+      </c>
+      <c r="D110" t="s">
+        <v>104</v>
+      </c>
+      <c r="E110" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>48</v>
+      </c>
+      <c r="B111" t="s">
         <v>62</v>
       </c>
-      <c r="C107" t="s">
+      <c r="C111" t="s">
+        <v>105</v>
+      </c>
+      <c r="D111" t="s">
+        <v>106</v>
+      </c>
+      <c r="E111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>48</v>
+      </c>
+      <c r="B112" t="s">
+        <v>62</v>
+      </c>
+      <c r="C112" t="s">
+        <v>107</v>
+      </c>
+      <c r="D112" t="s">
+        <v>108</v>
+      </c>
+      <c r="E112" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>48</v>
+      </c>
+      <c r="B113" t="s">
+        <v>62</v>
+      </c>
+      <c r="C113" t="s">
+        <v>109</v>
+      </c>
+      <c r="D113" t="s">
         <v>110</v>
       </c>
-      <c r="D107" t="s">
+      <c r="E113" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>48</v>
+      </c>
+      <c r="B114" t="s">
+        <v>62</v>
+      </c>
+      <c r="C114" t="s">
         <v>111</v>
       </c>
-      <c r="E107" t="n">
+      <c r="D114" t="s">
+        <v>112</v>
+      </c>
+      <c r="E114" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6097,19 +6213,19 @@
         <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I1" t="s">
         <v>16</v>
@@ -6125,10 +6241,10 @@
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G2"/>
       <c r="H2"/>
@@ -6145,7 +6261,7 @@
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G3"/>
       <c r="H3"/>
@@ -6162,7 +6278,7 @@
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
@@ -6175,12 +6291,12 @@
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6">
@@ -6188,18 +6304,18 @@
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H6"/>
       <c r="I6"/>
@@ -6209,18 +6325,18 @@
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H7"/>
       <c r="I7"/>
@@ -6230,18 +6346,18 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H8"/>
       <c r="I8"/>
@@ -6251,18 +6367,18 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
@@ -6272,18 +6388,18 @@
         <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H10"/>
       <c r="I10"/>
@@ -6293,18 +6409,18 @@
         <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H11"/>
       <c r="I11"/>
@@ -6314,18 +6430,18 @@
         <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H12"/>
       <c r="I12"/>
@@ -6335,18 +6451,18 @@
         <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E13"/>
       <c r="F13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H13"/>
       <c r="I13"/>
@@ -6356,18 +6472,18 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H14"/>
       <c r="I14"/>
@@ -6377,18 +6493,18 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E15"/>
       <c r="F15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H15"/>
       <c r="I15"/>
@@ -6398,18 +6514,18 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C16"/>
       <c r="D16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H16"/>
       <c r="I16"/>
@@ -6419,18 +6535,18 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E17"/>
       <c r="F17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H17"/>
       <c r="I17"/>
@@ -6440,18 +6556,18 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G18" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H18"/>
       <c r="I18"/>
@@ -6461,18 +6577,18 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G19" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H19"/>
       <c r="I19"/>
@@ -6482,18 +6598,18 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C20"/>
       <c r="D20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E20"/>
       <c r="F20" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G20" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H20"/>
       <c r="I20"/>
@@ -6503,18 +6619,18 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C21"/>
       <c r="D21" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E21"/>
       <c r="F21" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
@@ -6524,18 +6640,18 @@
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C22"/>
       <c r="D22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E22"/>
       <c r="F22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H22"/>
       <c r="I22"/>
@@ -6545,18 +6661,18 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C23"/>
       <c r="D23" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E23"/>
       <c r="F23" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H23"/>
       <c r="I23"/>
@@ -6570,7 +6686,7 @@
       <c r="D24"/>
       <c r="E24"/>
       <c r="F24" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G24"/>
       <c r="H24"/>
@@ -6581,18 +6697,18 @@
         <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C25"/>
       <c r="D25" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E25"/>
       <c r="F25" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H25"/>
       <c r="I25"/>
@@ -6602,18 +6718,18 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C26"/>
       <c r="D26" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E26"/>
       <c r="F26" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G26" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H26"/>
       <c r="I26"/>
@@ -6623,18 +6739,18 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C27"/>
       <c r="D27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E27"/>
       <c r="F27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G27" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H27"/>
       <c r="I27"/>
@@ -6644,18 +6760,18 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C28"/>
       <c r="D28" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E28"/>
       <c r="F28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H28"/>
       <c r="I28"/>
@@ -6665,18 +6781,18 @@
         <v>41</v>
       </c>
       <c r="B29" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E29"/>
       <c r="F29" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H29"/>
       <c r="I29"/>
@@ -6686,18 +6802,18 @@
         <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E30"/>
       <c r="F30" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G30" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H30"/>
       <c r="I30"/>
@@ -6707,18 +6823,18 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C31"/>
       <c r="D31" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E31"/>
       <c r="F31" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H31"/>
       <c r="I31"/>
@@ -6728,18 +6844,18 @@
         <v>48</v>
       </c>
       <c r="B32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C32"/>
       <c r="D32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E32"/>
       <c r="F32" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H32"/>
       <c r="I32"/>
@@ -6749,18 +6865,18 @@
         <v>48</v>
       </c>
       <c r="B33" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C33"/>
       <c r="D33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E33"/>
       <c r="F33" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H33"/>
       <c r="I33"/>
@@ -6770,18 +6886,18 @@
         <v>48</v>
       </c>
       <c r="B34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C34"/>
       <c r="D34" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E34"/>
       <c r="F34" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G34" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H34"/>
       <c r="I34"/>
@@ -6791,18 +6907,18 @@
         <v>48</v>
       </c>
       <c r="B35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C35"/>
       <c r="D35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E35"/>
       <c r="F35" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H35"/>
       <c r="I35"/>
@@ -6827,10 +6943,10 @@
         <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -6850,85 +6966,85 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="N1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="O1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Q1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="R1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="S1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="U1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="V1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="W1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="X1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Y1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Z1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AA1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AB1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AC1" t="s">
         <v>16</v>
@@ -6948,25 +7064,25 @@
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="O2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="Q2"/>
       <c r="R2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="S2"/>
       <c r="T2"/>
       <c r="U2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="V2"/>
       <c r="W2"/>
@@ -6976,7 +7092,7 @@
       <c r="AA2"/>
       <c r="AB2"/>
       <c r="AC2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3">
@@ -6984,10 +7100,10 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -7021,7 +7137,7 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -7056,10 +7172,10 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -7093,7 +7209,7 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -7128,10 +7244,10 @@
         <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -7165,7 +7281,7 @@
         <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -7200,7 +7316,7 @@
         <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
@@ -7235,7 +7351,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
@@ -7270,7 +7386,7 @@
         <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C11"/>
       <c r="D11"/>
@@ -7305,10 +7421,10 @@
         <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
@@ -7342,10 +7458,10 @@
         <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -7391,28 +7507,28 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -7421,10 +7537,10 @@
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -7447,104 +7563,104 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="I1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="Q1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="R1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="S1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="T1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="U1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="V1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="W1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="X1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="Y1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="Z1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AA1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AB1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AC1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AD1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AE1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AF1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>

</xml_diff>